<commit_message>
feat: make consent date required when consenting
</commit_message>
<xml_diff>
--- a/Criminal_Risk_Assessment_Request_XLSForm.xlsx
+++ b/Criminal_Risk_Assessment_Request_XLSForm.xlsx
@@ -637,10 +637,14 @@
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Date of consent is required.</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>not(selected(${is_unconsented}, 'unconsented'))</t>

</xml_diff>

<commit_message>
feat: make consent signature required when consenting
</commit_message>
<xml_diff>
--- a/Criminal_Risk_Assessment_Request_XLSForm.xlsx
+++ b/Criminal_Risk_Assessment_Request_XLSForm.xlsx
@@ -675,10 +675,14 @@
       <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Signature is required.</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>not(selected(${is_unconsented}, 'unconsented'))</t>

</xml_diff>

<commit_message>
fix: convert subject_name_header to read-only calculated field for ODK UI rendering
</commit_message>
<xml_diff>
--- a/Criminal_Risk_Assessment_Request_XLSForm.xlsx
+++ b/Criminal_Risk_Assessment_Request_XLSForm.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -530,6 +530,11 @@
           <t>calculation</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>read_only</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1403,7 +1408,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1413,11 +1418,14 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>NAME OF PERSON BEING ASSESSED: ${calc_full_name}
-*Must match information on page 1</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr"/>
+          <t>NAME OF PERSON BEING ASSESSED:</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>*Must match information on page 1</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3" t="inlineStr"/>
       <c r="G30" s="3" t="inlineStr"/>
@@ -1425,7 +1433,16 @@
       <c r="I30" s="3" t="inlineStr"/>
       <c r="J30" s="3" t="inlineStr"/>
       <c r="K30" s="3" t="inlineStr"/>
-      <c r="L30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>${calc_full_name}</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">

</xml_diff>